<commit_message>
chore: run 2026-03-28 21:05 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_28_03_2026.xlsx
+++ b/logs/Consolidado_28_03_2026.xlsx
@@ -679,7 +679,7 @@
         <v>15</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>5</v>
@@ -755,7 +755,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -20065,11 +20065,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>7757309</t>
-        </is>
-      </c>
+      <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>20%</t>

</xml_diff>